<commit_message>
M3.2: XLSX geometry — real column widths, row heights, merged cells
Self-written OOXML geometry parser (dv-xlsx/model.rs, quick-xml + zip):
- column widths (<cols>) and row heights (<row ht>)
- merged cells (<mergeCells>): cover interior grid lines + redraw outer border,
  span the anchor cell's text across the region
- variable-width/height grid via prefix-sum column/row boundaries

Values still via calamine; verified natively and in-browser (merged title +
varied widths on the 繁中 sample).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/assets/sample.xlsx
+++ b/examples/assets/sample.xlsx
@@ -8,7 +8,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+  <si>
+    <t>2024 年水果銷售統計表</t>
+  </si>
   <si>
     <t>產品</t>
   </si>
@@ -41,37 +44,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="9" customWidth="1"/>
+    <col min="3" max="3" width="9" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
         <v>4</v>
-      </c>
-      <c r="B2">
-        <v>10</v>
-      </c>
-      <c r="C2">
-        <v>35</v>
-      </c>
-      <c r="D2">
-        <v>350</v>
       </c>
     </row>
     <row r="3">
@@ -79,13 +76,13 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C3">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="D3">
-        <v>360</v>
+        <v>350</v>
       </c>
     </row>
     <row r="4">
@@ -93,13 +90,13 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C4">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="D4">
-        <v>375</v>
+        <v>360</v>
       </c>
     </row>
     <row r="5">
@@ -107,13 +104,13 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="C5">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="D5">
-        <v>480</v>
+        <v>375</v>
       </c>
     </row>
     <row r="6">
@@ -121,12 +118,29 @@
         <v>8</v>
       </c>
       <c r="B6">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>60</v>
+      </c>
+      <c r="D6">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
         <v>53</v>
       </c>
-      <c r="D6">
+      <c r="D7">
         <v>1565</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
M3.3: XLSX styles — fills, fonts, borders, alignment, number formats
OOXML styles.xml parser (fonts/fills/borders/numFmts/cellXfs + per-cell xf) and
a pragmatic number-format engine:
- solid fills (rgb + theme palette w/ tint), font bold + colour, cell borders,
  horizontal alignment
- number formats: thousands grouping, decimals, percent, currency ($), and
  Excel-serial dates (1900 system)
- faux-bold in dv-render (stroke glyph outlines; one font face loaded)

Verified natively + in-browser: styled 繁中 sheet (blue title, bold header,
borders, $5,280 / $6,365 currency, bold totals).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/assets/sample.xlsx
+++ b/examples/assets/sample.xlsx
@@ -42,6 +42,93 @@
 </sst>
 </file>
 
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="#,##0"/>
+    <numFmt numFmtId="165" formatCode="$#,##0"/>
+  </numFmts>
+  <fonts count="3">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+    </font>
+  </fonts>
+  <fills count="4">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4F81BD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E1F2"/>
+      </patternFill>
+    </fill>
+  </fills>
+  <borders count="3">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+</styleSheet>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:D7"/>
@@ -49,93 +136,93 @@
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
     <col min="3" max="3" width="9" customWidth="1"/>
-    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s">
+      <c r="A3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="3">
         <v>10</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="3">
         <v>35</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="4">
         <v>350</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s">
+      <c r="A4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="3">
         <v>20</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="3">
         <v>18</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="4">
         <v>360</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s">
+      <c r="A5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="3">
         <v>15</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="3">
         <v>25</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="4">
         <v>375</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s">
+      <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B6">
-        <v>8</v>
-      </c>
-      <c r="C6">
+      <c r="B6" s="3">
+        <v>88</v>
+      </c>
+      <c r="C6" s="3">
         <v>60</v>
       </c>
-      <c r="D6">
-        <v>480</v>
+      <c r="D6" s="4">
+        <v>5280</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s">
+      <c r="A7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B7">
-        <v>53</v>
-      </c>
-      <c r="D7">
-        <v>1565</v>
+      <c r="B7" s="6">
+        <v>133</v>
+      </c>
+      <c r="D7" s="7">
+        <v>6365</v>
       </c>
     </row>
   </sheetData>

</xml_diff>